<commit_message>
refactor: modbus runner 改为 round-robin 单请求调度器，更新鸿合配置
- runner: 移除 poll_interval / flush_priority_writes / read_blocks / drain_downlinks，
  改为单请求 round-robin 调度器（drain_writes_nb + request_one 逐块轮询），
  写延迟 ≤ request_interval 且不随块数增长
- mqtt: 鸿合项目 topic bank 前缀映射为 bcu
- config: 更新鸿合 BMS 与总配置，新增水冷机组/消防温感烟感/除湿机配置

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/鸿合_配置_v2.0.xlsx
+++ b/config/鸿合_配置_v2.0.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="18519" windowHeight="11218" activeTab="3"/>
+    <workbookView windowWidth="18569" windowHeight="10825" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="project" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="204">
   <si>
     <t>key</t>
   </si>
@@ -253,6 +253,9 @@
     <t>maxGap</t>
   </si>
   <si>
+    <t>pcs</t>
+  </si>
+  <si>
     <t>ModbusTCP</t>
   </si>
   <si>
@@ -262,37 +265,31 @@
     <t>192.168.0.1</t>
   </si>
   <si>
+    <t>bms</t>
+  </si>
+  <si>
     <t>192.168.0.2</t>
   </si>
   <si>
+    <t>tms</t>
+  </si>
+  <si>
     <t>192.168.0.3</t>
   </si>
   <si>
+    <t>dehum</t>
+  </si>
+  <si>
     <t>192.168.0.4</t>
   </si>
   <si>
+    <t>fire</t>
+  </si>
+  <si>
     <t>./config/BMS_鸿合国轩.xlsx</t>
   </si>
   <si>
     <t>192.168.0.6</t>
-  </si>
-  <si>
-    <t>192.168.0.7</t>
-  </si>
-  <si>
-    <t>192.168.0.8</t>
-  </si>
-  <si>
-    <t>192.168.0.9</t>
-  </si>
-  <si>
-    <t>IEC104</t>
-  </si>
-  <si>
-    <t>./config/测控柜_鸿合.xlsx</t>
-  </si>
-  <si>
-    <t>192.168.0.5</t>
   </si>
   <si>
     <t>device_id</t>
@@ -1299,7 +1296,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1317,9 +1314,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center" vertical="center"/>
@@ -9089,8 +9083,8 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:S10"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18"/>
+  <dimension ref="A1:S6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelRow="5"/>
   <cols>
     <col min="1" max="1" width="6.46031746031746" style="2" customWidth="1"/>
     <col min="2" max="2" width="15.5952380952381" style="2" customWidth="1"/>
@@ -9172,16 +9166,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>43</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F2" s="2">
         <v>1000</v>
@@ -9190,7 +9184,7 @@
         <v>1000</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I2" s="2">
         <v>502</v>
@@ -9208,16 +9202,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>45</v>
+        <v>76</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>43</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F3" s="2">
         <v>1000</v>
@@ -9226,7 +9220,7 @@
         <v>1000</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I3" s="2">
         <v>502</v>
@@ -9244,16 +9238,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>46</v>
+        <v>78</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>43</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F4" s="2">
         <v>1000</v>
@@ -9262,7 +9256,7 @@
         <v>1000</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I4" s="2">
         <v>502</v>
@@ -9280,16 +9274,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>47</v>
+        <v>80</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>43</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F5" s="2">
         <v>1000</v>
@@ -9298,7 +9292,7 @@
         <v>1000</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="I5" s="2">
         <v>502</v>
@@ -9316,16 +9310,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>48</v>
+        <v>82</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>49</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="F6" s="2">
         <v>1000</v>
@@ -9334,7 +9328,7 @@
         <v>5000</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I6" s="2">
         <v>502</v>
@@ -9344,137 +9338,6 @@
       </c>
       <c r="S6" s="2">
         <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19">
-      <c r="A7" s="2">
-        <f>devices!A7</f>
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F7" s="2">
-        <v>1000</v>
-      </c>
-      <c r="G7" s="2">
-        <v>5000</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="I7" s="2">
-        <v>502</v>
-      </c>
-      <c r="J7" s="2">
-        <v>1</v>
-      </c>
-      <c r="S7" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19">
-      <c r="A8" s="2">
-        <f>devices!A8</f>
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F8" s="2">
-        <v>1000</v>
-      </c>
-      <c r="G8" s="2">
-        <v>5000</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="I8" s="2">
-        <v>502</v>
-      </c>
-      <c r="J8" s="2">
-        <v>1</v>
-      </c>
-      <c r="S8" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19">
-      <c r="A9" s="2">
-        <f>devices!A9</f>
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F9" s="2">
-        <v>1000</v>
-      </c>
-      <c r="G9" s="2">
-        <v>5000</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="I9" s="2">
-        <v>502</v>
-      </c>
-      <c r="J9" s="2">
-        <v>1</v>
-      </c>
-      <c r="S9" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19">
-      <c r="A10" s="2">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="I10" s="2">
-        <v>2404</v>
       </c>
     </row>
   </sheetData>
@@ -9501,16 +9364,16 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:7">
       <c r="A1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>89</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -9521,7 +9384,7 @@
         <v>42</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C2" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[1]遥测!$A$56:$A$71)&amp;",65535"</f>
@@ -9536,7 +9399,7 @@
         <v>42</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C3" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[1]遥测!$A$2:$A$55)</f>
@@ -9551,7 +9414,7 @@
         <v>42</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C4" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[1]遥调!$A$2:$A$31)</f>
@@ -9566,7 +9429,7 @@
         <v>45</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C5" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[1]遥测!$A$56:$A$71)&amp;",65535"</f>
@@ -9581,10 +9444,10 @@
         <v>45</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>94</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>95</v>
       </c>
       <c r="D6" s="3">
         <v>1</v>
@@ -9595,10 +9458,10 @@
         <v>45</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>96</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>97</v>
       </c>
       <c r="D7" s="3">
         <v>1</v>
@@ -9609,7 +9472,7 @@
         <v>46</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C8" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[1]遥测!$A$56:$A$71)&amp;",65535"</f>
@@ -9624,10 +9487,10 @@
         <v>46</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D9" s="3">
         <v>1</v>
@@ -9638,10 +9501,10 @@
         <v>46</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D10" s="3">
         <v>1</v>
@@ -9652,7 +9515,7 @@
         <v>47</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C11" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[1]遥测!$A$56:$A$71)&amp;",65535"</f>
@@ -9667,10 +9530,10 @@
         <v>47</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D12" s="3">
         <v>1</v>
@@ -9681,10 +9544,10 @@
         <v>47</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D13" s="3">
         <v>1</v>
@@ -9695,7 +9558,7 @@
         <v>48</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C14" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$2:$A$141,[3]遥测!$A$300:$A$317)&amp;",65535"</f>
@@ -9710,7 +9573,7 @@
         <v>48</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C15" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥测!$A$2:$A$53)</f>
@@ -9725,7 +9588,7 @@
         <v>48</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C16" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥调!$A$2:$A$20)</f>
@@ -9740,7 +9603,7 @@
         <v>51</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C17" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$2:$A$141,[3]遥测!$A$300:$A$317)&amp;",65535"</f>
@@ -9755,7 +9618,7 @@
         <v>51</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C18" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥测!$A$2:$A$53)</f>
@@ -9770,7 +9633,7 @@
         <v>51</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C19" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥调!$A$2:$A$20)</f>
@@ -9785,7 +9648,7 @@
         <v>52</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C20" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$2:$A$141,[3]遥测!$A$300:$A$317)&amp;",65535"</f>
@@ -9800,10 +9663,10 @@
         <v>52</v>
       </c>
       <c r="B21" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C21" s="3" t="s">
         <v>111</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>112</v>
       </c>
       <c r="D21" s="3">
         <v>1</v>
@@ -9814,10 +9677,10 @@
         <v>52</v>
       </c>
       <c r="B22" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C22" s="3" t="s">
         <v>113</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>114</v>
       </c>
       <c r="D22" s="3">
         <v>1</v>
@@ -9828,7 +9691,7 @@
         <v>53</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C23" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$2:$A$141,[3]遥测!$A$300:$A$317)&amp;",65535"</f>
@@ -9843,10 +9706,10 @@
         <v>53</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D24" s="3">
         <v>1</v>
@@ -9857,10 +9720,10 @@
         <v>53</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D25" s="3">
         <v>1</v>
@@ -9871,7 +9734,7 @@
         <v>48</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C26" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥测!$A$54:$A$92)</f>
@@ -9886,7 +9749,7 @@
         <v>48</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C27" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥测!$A$93:$A$131)</f>
@@ -9901,7 +9764,7 @@
         <v>48</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C28" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥测!$A$132:$A$170)</f>
@@ -9916,7 +9779,7 @@
         <v>48</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C29" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥测!$A$171:$A$209)</f>
@@ -9931,7 +9794,7 @@
         <v>48</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C30" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥测!$A$210:$A$248)</f>
@@ -9946,7 +9809,7 @@
         <v>48</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C31" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥测!$A$249:$A$287)</f>
@@ -9961,10 +9824,10 @@
         <v>51</v>
       </c>
       <c r="B32" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C32" s="3" t="s">
         <v>124</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>125</v>
       </c>
       <c r="D32" s="3">
         <v>1</v>
@@ -9975,10 +9838,10 @@
         <v>51</v>
       </c>
       <c r="B33" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C33" s="3" t="s">
         <v>126</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>127</v>
       </c>
       <c r="D33" s="3">
         <v>1</v>
@@ -9989,10 +9852,10 @@
         <v>51</v>
       </c>
       <c r="B34" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C34" s="3" t="s">
         <v>128</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>129</v>
       </c>
       <c r="D34" s="3">
         <v>1</v>
@@ -10003,10 +9866,10 @@
         <v>51</v>
       </c>
       <c r="B35" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C35" s="3" t="s">
         <v>130</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>131</v>
       </c>
       <c r="D35" s="3">
         <v>1</v>
@@ -10017,10 +9880,10 @@
         <v>51</v>
       </c>
       <c r="B36" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C36" s="3" t="s">
         <v>132</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>133</v>
       </c>
       <c r="D36" s="3">
         <v>1</v>
@@ -10031,10 +9894,10 @@
         <v>51</v>
       </c>
       <c r="B37" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C37" s="3" t="s">
         <v>134</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>135</v>
       </c>
       <c r="D37" s="3">
         <v>1</v>
@@ -10045,7 +9908,7 @@
         <v>52</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C38" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥测!$A$54:$A$92)</f>
@@ -10060,7 +9923,7 @@
         <v>52</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C39" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥测!$A$93:$A$131)</f>
@@ -10075,7 +9938,7 @@
         <v>52</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C40" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥测!$A$132:$A$170)</f>
@@ -10090,7 +9953,7 @@
         <v>52</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C41" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥测!$A$171:$A$209)</f>
@@ -10105,7 +9968,7 @@
         <v>52</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C42" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥测!$A$210:$A$248)</f>
@@ -10120,7 +9983,7 @@
         <v>52</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C43" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥测!$A$249:$A$287)</f>
@@ -10135,10 +9998,10 @@
         <v>53</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D44" s="3">
         <v>1</v>
@@ -10149,10 +10012,10 @@
         <v>53</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D45" s="3">
         <v>1</v>
@@ -10163,10 +10026,10 @@
         <v>53</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D46" s="3">
         <v>1</v>
@@ -10177,10 +10040,10 @@
         <v>53</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D47" s="3">
         <v>1</v>
@@ -10191,10 +10054,10 @@
         <v>53</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D48" s="3">
         <v>1</v>
@@ -10205,10 +10068,10 @@
         <v>53</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="C49" s="7" t="s">
-        <v>135</v>
+        <v>146</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>134</v>
       </c>
       <c r="D49" s="3">
         <v>1</v>
@@ -10219,10 +10082,10 @@
         <v>48</v>
       </c>
       <c r="B50" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C50" s="4" t="s">
         <v>148</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>149</v>
       </c>
       <c r="D50" s="3">
         <v>1</v>
@@ -10233,10 +10096,10 @@
         <v>48</v>
       </c>
       <c r="B51" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C51" s="4" t="s">
         <v>150</v>
-      </c>
-      <c r="C51" s="4" t="s">
-        <v>151</v>
       </c>
       <c r="D51" s="3">
         <v>1</v>
@@ -10247,10 +10110,10 @@
         <v>48</v>
       </c>
       <c r="B52" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C52" s="4" t="s">
         <v>152</v>
-      </c>
-      <c r="C52" s="4" t="s">
-        <v>153</v>
       </c>
       <c r="D52" s="3">
         <v>1</v>
@@ -10261,10 +10124,10 @@
         <v>48</v>
       </c>
       <c r="B53" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C53" s="4" t="s">
         <v>154</v>
-      </c>
-      <c r="C53" s="4" t="s">
-        <v>155</v>
       </c>
       <c r="D53" s="3">
         <v>1</v>
@@ -10275,10 +10138,10 @@
         <v>48</v>
       </c>
       <c r="B54" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C54" s="4" t="s">
         <v>156</v>
-      </c>
-      <c r="C54" s="4" t="s">
-        <v>157</v>
       </c>
       <c r="D54" s="3">
         <v>1</v>
@@ -10289,10 +10152,10 @@
         <v>48</v>
       </c>
       <c r="B55" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C55" s="4" t="s">
         <v>158</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>159</v>
       </c>
       <c r="D55" s="3">
         <v>1</v>
@@ -10303,10 +10166,10 @@
         <v>51</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D56" s="3">
         <v>1</v>
@@ -10317,10 +10180,10 @@
         <v>51</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D57" s="3">
         <v>1</v>
@@ -10331,10 +10194,10 @@
         <v>51</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D58" s="3">
         <v>1</v>
@@ -10345,10 +10208,10 @@
         <v>51</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D59" s="3">
         <v>1</v>
@@ -10359,10 +10222,10 @@
         <v>51</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D60" s="3">
         <v>1</v>
@@ -10373,10 +10236,10 @@
         <v>51</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D61" s="3">
         <v>1</v>
@@ -10387,10 +10250,10 @@
         <v>52</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D62" s="3">
         <v>1</v>
@@ -10401,10 +10264,10 @@
         <v>52</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D63" s="3">
         <v>1</v>
@@ -10415,10 +10278,10 @@
         <v>52</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D64" s="3">
         <v>1</v>
@@ -10429,10 +10292,10 @@
         <v>52</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D65" s="3">
         <v>1</v>
@@ -10443,10 +10306,10 @@
         <v>52</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D66" s="3">
         <v>1</v>
@@ -10457,10 +10320,10 @@
         <v>52</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D67" s="3">
         <v>1</v>
@@ -10471,10 +10334,10 @@
         <v>53</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D68" s="3">
         <v>1</v>
@@ -10485,10 +10348,10 @@
         <v>53</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D69" s="3">
         <v>1</v>
@@ -10499,10 +10362,10 @@
         <v>53</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D70" s="3">
         <v>1</v>
@@ -10513,10 +10376,10 @@
         <v>53</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D71" s="3">
         <v>1</v>
@@ -10527,10 +10390,10 @@
         <v>53</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D72" s="3">
         <v>1</v>
@@ -10541,10 +10404,10 @@
         <v>53</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D73" s="3">
         <v>1</v>
@@ -10555,7 +10418,7 @@
         <v>48</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C74" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$142:$A$256)</f>
@@ -10570,7 +10433,7 @@
         <v>48</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C75" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$257:$A$371)</f>
@@ -10585,7 +10448,7 @@
         <v>48</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C76" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$372:$A$486)</f>
@@ -10600,7 +10463,7 @@
         <v>48</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C77" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$487:$A$601)</f>
@@ -10615,7 +10478,7 @@
         <v>48</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C78" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$602:$A$716)</f>
@@ -10630,7 +10493,7 @@
         <v>48</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C79" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$717:$A$831)</f>
@@ -10645,7 +10508,7 @@
         <v>51</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C80" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$142:$A$256)</f>
@@ -10660,7 +10523,7 @@
         <v>51</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C81" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$257:$A$371)</f>
@@ -10675,7 +10538,7 @@
         <v>51</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C82" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$372:$A$486)</f>
@@ -10690,7 +10553,7 @@
         <v>51</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C83" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$487:$A$601)</f>
@@ -10705,7 +10568,7 @@
         <v>51</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C84" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$602:$A$716)</f>
@@ -10720,7 +10583,7 @@
         <v>51</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C85" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$717:$A$831)</f>
@@ -10735,7 +10598,7 @@
         <v>52</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C86" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$142:$A$256)</f>
@@ -10750,7 +10613,7 @@
         <v>52</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C87" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$257:$A$371)</f>
@@ -10765,7 +10628,7 @@
         <v>52</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C88" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$372:$A$486)</f>
@@ -10780,7 +10643,7 @@
         <v>52</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C89" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$487:$A$601)</f>
@@ -10795,7 +10658,7 @@
         <v>52</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C90" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$602:$A$716)</f>
@@ -10810,7 +10673,7 @@
         <v>52</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C91" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$717:$A$831)</f>
@@ -10825,7 +10688,7 @@
         <v>53</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C92" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$142:$A$256)</f>
@@ -10840,7 +10703,7 @@
         <v>53</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C93" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$257:$A$371)</f>
@@ -10855,7 +10718,7 @@
         <v>53</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C94" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$372:$A$486)</f>
@@ -10870,7 +10733,7 @@
         <v>53</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C95" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$487:$A$601)</f>
@@ -10885,7 +10748,7 @@
         <v>53</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C96" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$602:$A$716)</f>
@@ -10900,7 +10763,7 @@
         <v>53</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C97" s="3" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[3]遥信!$A$717:$A$831)</f>
@@ -10915,7 +10778,7 @@
         <v>54</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C98" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[2]遥信!$A$2:$A$120)&amp;",65535"</f>
@@ -10930,7 +10793,7 @@
         <v>54</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C99" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[2]遥测!$A$2:$A$200)</f>
@@ -10945,7 +10808,7 @@
         <v>54</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C100" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[2]遥控!$A$2:$A$120)</f>

</xml_diff>